<commit_message>
Add project Excel files
</commit_message>
<xml_diff>
--- a/deadline_laptrinhmang.xlsx
+++ b/deadline_laptrinhmang.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\GITHUB\UDM_05\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D7D65492-5E06-43E8-86E6-CDD46F491974}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D8C48197-5B2E-4677-BAAC-E2ECE6591770}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{4996BFC1-5545-47D6-BEAA-54FAD06ABAD6}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="165" uniqueCount="84">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="165" uniqueCount="83">
   <si>
     <t>STT</t>
   </si>
@@ -55,9 +55,6 @@
   </si>
   <si>
     <t>Architecture &amp; Protocol</t>
-  </si>
-  <si>
-    <t>Nguyễn Hoàng Phúc</t>
   </si>
   <si>
     <r>
@@ -1354,19 +1351,19 @@
         <v>9</v>
       </c>
       <c r="D2" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="E2" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="E2" s="2" t="s">
+      <c r="F2" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="F2" s="2" t="s">
-        <v>12</v>
-      </c>
       <c r="G2" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="H2" s="2" t="s">
         <v>13</v>
-      </c>
-      <c r="H2" s="2" t="s">
-        <v>14</v>
       </c>
     </row>
     <row r="3" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -1377,22 +1374,22 @@
         <v>8</v>
       </c>
       <c r="C3" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="D3" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="D3" s="2" t="s">
+      <c r="E3" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="E3" s="2" t="s">
+      <c r="F3" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="G3" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="H3" s="2" t="s">
         <v>17</v>
-      </c>
-      <c r="F3" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="G3" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="H3" s="2" t="s">
-        <v>18</v>
       </c>
     </row>
     <row r="4" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -1403,22 +1400,22 @@
         <v>8</v>
       </c>
       <c r="C4" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D4" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="D4" s="2" t="s">
+      <c r="E4" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="E4" s="2" t="s">
-        <v>21</v>
-      </c>
       <c r="F4" s="2" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="H4" s="2" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
     <row r="5" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -1429,19 +1426,19 @@
         <v>8</v>
       </c>
       <c r="C5" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="D5" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="D5" s="2" t="s">
+      <c r="E5" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="E5" s="2" t="s">
-        <v>24</v>
-      </c>
       <c r="F5" s="2" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="G5" s="3" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="H5" s="2"/>
     </row>
@@ -1453,19 +1450,19 @@
         <v>8</v>
       </c>
       <c r="C6" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="D6" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="D6" s="2" t="s">
+      <c r="E6" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="E6" s="2" t="s">
-        <v>27</v>
-      </c>
       <c r="F6" s="2" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="G6" s="3" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="H6" s="2"/>
     </row>
@@ -1477,19 +1474,19 @@
         <v>8</v>
       </c>
       <c r="C7" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="D7" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="D7" s="2" t="s">
+      <c r="E7" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="E7" s="2" t="s">
-        <v>31</v>
-      </c>
       <c r="F7" s="2" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="G7" s="3" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="H7" s="2"/>
     </row>
@@ -1498,22 +1495,22 @@
         <v>7</v>
       </c>
       <c r="B8" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="C8" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="C8" s="1" t="s">
+      <c r="D8" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="E8" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="D8" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="E8" s="2" t="s">
+      <c r="F8" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="F8" s="2" t="s">
-        <v>35</v>
-      </c>
       <c r="G8" s="3" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="H8" s="2"/>
     </row>
@@ -1522,22 +1519,22 @@
         <v>8</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C9" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="E9" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="D9" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="E9" s="2" t="s">
-        <v>37</v>
-      </c>
       <c r="F9" s="2" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="G9" s="3" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="H9" s="2"/>
     </row>
@@ -1546,25 +1543,25 @@
         <v>9</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C10" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="E10" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="D10" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="E10" s="2" t="s">
-        <v>39</v>
-      </c>
       <c r="F10" s="2" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="G10" s="3" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="H10" s="2" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
     <row r="11" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -1572,22 +1569,22 @@
         <v>10</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C11" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="D11" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="E11" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="D11" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="E11" s="2" t="s">
-        <v>41</v>
-      </c>
       <c r="F11" s="2" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="G11" s="3" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="H11" s="2"/>
     </row>
@@ -1596,22 +1593,22 @@
         <v>11</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C12" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="D12" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="E12" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="D12" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="E12" s="2" t="s">
-        <v>43</v>
-      </c>
       <c r="F12" s="2" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="G12" s="3" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="H12" s="2"/>
     </row>
@@ -1620,22 +1617,22 @@
         <v>12</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C13" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="D13" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="E13" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="D13" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="E13" s="2" t="s">
-        <v>45</v>
-      </c>
       <c r="F13" s="2" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="G13" s="3" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="H13" s="2"/>
     </row>
@@ -1644,22 +1641,22 @@
         <v>13</v>
       </c>
       <c r="B14" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="C14" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="C14" s="1" t="s">
+      <c r="D14" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="E14" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="D14" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="E14" s="2" t="s">
+      <c r="F14" s="4" t="s">
         <v>48</v>
       </c>
-      <c r="F14" s="4" t="s">
-        <v>49</v>
-      </c>
       <c r="G14" s="3" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="H14" s="2"/>
     </row>
@@ -1668,25 +1665,25 @@
         <v>14</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C15" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="D15" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="E15" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="D15" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="E15" s="2" t="s">
-        <v>51</v>
-      </c>
       <c r="F15" s="4" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="G15" s="3" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="H15" s="2" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
     </row>
     <row r="16" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -1694,22 +1691,22 @@
         <v>15</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C16" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="D16" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="E16" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="D16" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="E16" s="2" t="s">
-        <v>53</v>
-      </c>
       <c r="F16" s="4" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="G16" s="3" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="H16" s="2"/>
     </row>
@@ -1718,22 +1715,22 @@
         <v>16</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C17" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="D17" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="E17" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="D17" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="E17" s="2" t="s">
-        <v>55</v>
-      </c>
       <c r="F17" s="4" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="G17" s="3" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="H17" s="2"/>
     </row>
@@ -1742,22 +1739,22 @@
         <v>17</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C18" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="D18" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="E18" s="2" t="s">
         <v>56</v>
       </c>
-      <c r="D18" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="E18" s="2" t="s">
-        <v>57</v>
-      </c>
       <c r="F18" s="4" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="G18" s="3" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="H18" s="2"/>
     </row>
@@ -1766,22 +1763,22 @@
         <v>18</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C19" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="D19" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="E19" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="D19" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="E19" s="2" t="s">
-        <v>59</v>
-      </c>
       <c r="F19" s="4" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="G19" s="3" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="H19" s="2"/>
     </row>
@@ -1790,25 +1787,25 @@
         <v>19</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="D20" s="2" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="E20" s="2" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="F20" s="4">
         <v>46151</v>
       </c>
       <c r="G20" s="3" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="H20" s="2" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="21" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -1816,22 +1813,22 @@
         <v>20</v>
       </c>
       <c r="B21" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="C21" s="1" t="s">
         <v>60</v>
       </c>
-      <c r="C21" s="1" t="s">
+      <c r="D21" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="E21" s="2" t="s">
         <v>61</v>
-      </c>
-      <c r="D21" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="E21" s="2" t="s">
-        <v>62</v>
       </c>
       <c r="F21" s="4">
         <v>46151</v>
       </c>
       <c r="G21" s="3" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="H21" s="2"/>
     </row>
@@ -1840,22 +1837,22 @@
         <v>21</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C22" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="D22" s="2" t="s">
         <v>63</v>
       </c>
-      <c r="D22" s="2" t="s">
+      <c r="E22" s="2" t="s">
         <v>64</v>
-      </c>
-      <c r="E22" s="2" t="s">
-        <v>65</v>
       </c>
       <c r="F22" s="4">
         <v>46151</v>
       </c>
       <c r="G22" s="3" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="H22" s="2"/>
     </row>
@@ -1864,22 +1861,22 @@
         <v>22</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C23" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="D23" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="E23" s="2" t="s">
         <v>66</v>
-      </c>
-      <c r="D23" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="E23" s="2" t="s">
-        <v>67</v>
       </c>
       <c r="F23" s="4">
         <v>46151</v>
       </c>
       <c r="G23" s="3" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="H23" s="2"/>
     </row>
@@ -1888,22 +1885,22 @@
         <v>23</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C24" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="D24" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="E24" s="2" t="s">
         <v>68</v>
-      </c>
-      <c r="D24" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="E24" s="2" t="s">
-        <v>69</v>
       </c>
       <c r="F24" s="4">
         <v>46151</v>
       </c>
       <c r="G24" s="3" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="H24" s="2"/>
     </row>
@@ -1912,22 +1909,22 @@
         <v>24</v>
       </c>
       <c r="B25" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="C25" s="1" t="s">
         <v>70</v>
       </c>
-      <c r="C25" s="1" t="s">
+      <c r="D25" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="E25" s="2" t="s">
         <v>71</v>
-      </c>
-      <c r="D25" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="E25" s="2" t="s">
-        <v>72</v>
       </c>
       <c r="F25" s="4">
         <v>46365</v>
       </c>
       <c r="G25" s="3" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="H25" s="2"/>
     </row>
@@ -1936,22 +1933,22 @@
         <v>25</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="C26" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="D26" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="E26" s="2" t="s">
         <v>73</v>
-      </c>
-      <c r="D26" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="E26" s="2" t="s">
-        <v>74</v>
       </c>
       <c r="F26" s="4">
         <v>46365</v>
       </c>
       <c r="G26" s="3" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="H26" s="2"/>
     </row>
@@ -1960,38 +1957,38 @@
         <v>26</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="C27" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="D27" s="2" t="s">
         <v>75</v>
       </c>
-      <c r="D27" s="2" t="s">
+      <c r="E27" s="2" t="s">
         <v>76</v>
-      </c>
-      <c r="E27" s="2" t="s">
-        <v>77</v>
       </c>
       <c r="F27" s="4">
         <v>46365</v>
       </c>
       <c r="G27" s="3" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="H27" s="2"/>
     </row>
     <row r="64" spans="16:16" x14ac:dyDescent="0.3">
       <c r="P64" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
     </row>
     <row r="65" spans="16:16" x14ac:dyDescent="0.3">
       <c r="P65" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
     </row>
     <row r="66" spans="16:16" x14ac:dyDescent="0.3">
       <c r="P66" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
   </sheetData>

</xml_diff>